<commit_message>
style: simplify v0.10.0 workbook colors
</commit_message>
<xml_diff>
--- a/outputs/01a0b000-cf04-7f00-a568-1f20935b5dd8/vgb-property-calculation-advanced-v0.10.0-rescored.xlsx
+++ b/outputs/01a0b000-cf04-7f00-a568-1f20935b5dd8/vgb-property-calculation-advanced-v0.10.0-rescored.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作表 1" sheetId="1" r:id="R1d77e86e9bd4422f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作表 1" sheetId="1" r:id="Rfbbbd21db94e49aa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +17,7 @@
     <x:numFmt numFmtId="164" formatCode="0.000000"/>
     <x:numFmt numFmtId="165" formatCode="0.######"/>
   </x:numFmts>
-  <x:fonts count="14">
+  <x:fonts count="15">
     <x:font>
       <x:sz val="10"/>
       <x:color indexed="8"/>
@@ -96,8 +96,13 @@
       <x:color rgb="FF00FFFF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="18">
+  <x:fills count="23">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -184,8 +189,33 @@
         <x:fgColor rgb="FF000080"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4B5563"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE5E7EB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F4F6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD1D5DB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="28">
+  <x:borders count="30">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -526,13 +556,41 @@
         <x:color rgb="FF008000"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD1D5DB"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF9CA3AF"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF9CA3AF"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF9CA3AF"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF9CA3AF"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="230">
+  <x:cellXfs count="269">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
@@ -1206,6 +1264,123 @@
     </x:xf>
     <x:xf numFmtId="165" fontId="11" fillId="17" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="18" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="18" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="19" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="19" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="19" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="20" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="20" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="20" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="20" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="20" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="20" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="21" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="21" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="21" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="21" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="21" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="21" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="22" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="22" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="22" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="22" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="22" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="22" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="22" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="12" fillId="22" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="14" fillId="22" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="14" fillId="22" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="12" fillId="22" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="14" fillId="22" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="14" fillId="22" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="19" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="19" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="19" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="19" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="19" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="19" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="11" fillId="19" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="8" fillId="19" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="8" fillId="19" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1449,823 +1624,823 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" s="105" customFormat="1" ht="24" customHeight="1">
-      <x:c r="A1" s="130" t="str">
+      <x:c r="A1" s="231" t="str">
         <x:v>表格 1</x:v>
       </x:c>
-      <x:c r="B1" s="130"/>
-      <x:c r="C1" s="130"/>
-      <x:c r="D1" s="130"/>
-      <x:c r="E1" s="130"/>
-      <x:c r="F1" s="130"/>
-      <x:c r="G1" s="130"/>
-      <x:c r="H1" s="130"/>
-      <x:c r="I1" s="130"/>
-      <x:c r="J1" s="130"/>
-      <x:c r="K1" s="130"/>
+      <x:c r="B1" s="231"/>
+      <x:c r="C1" s="231"/>
+      <x:c r="D1" s="231"/>
+      <x:c r="E1" s="231"/>
+      <x:c r="F1" s="231"/>
+      <x:c r="G1" s="231"/>
+      <x:c r="H1" s="231"/>
+      <x:c r="I1" s="231"/>
+      <x:c r="J1" s="231"/>
+      <x:c r="K1" s="231"/>
     </x:row>
     <x:row r="2" s="105" customFormat="1" ht="30" customHeight="1">
-      <x:c r="A2" s="142" t="str">
+      <x:c r="A2" s="234" t="str">
         <x:v>题目 ID + 一句话概括</x:v>
       </x:c>
-      <x:c r="B2" s="142" t="str">
+      <x:c r="B2" s="234" t="str">
         <x:v>v0.10.0 容差范围</x:v>
       </x:c>
-      <x:c r="C2" s="142" t="str">
+      <x:c r="C2" s="234" t="str">
         <x:v>本题的标准答案</x:v>
       </x:c>
-      <x:c r="D2" s="142" t="str">
+      <x:c r="D2" s="234" t="str">
         <x:v>gpt-5-6-sol</x:v>
       </x:c>
-      <x:c r="E2" s="142"/>
-      <x:c r="F2" s="142" t="str">
+      <x:c r="E2" s="234"/>
+      <x:c r="F2" s="234" t="str">
         <x:v>gpt-5-6-sol</x:v>
       </x:c>
-      <x:c r="G2" s="142"/>
-      <x:c r="H2" s="142" t="str">
+      <x:c r="G2" s="234"/>
+      <x:c r="H2" s="234" t="str">
         <x:v>qwen3-8-flash</x:v>
       </x:c>
-      <x:c r="I2" s="142"/>
-      <x:c r="J2" s="142" t="str">
+      <x:c r="I2" s="234"/>
+      <x:c r="J2" s="234" t="str">
         <x:v>qwen3-8-flash</x:v>
       </x:c>
-      <x:c r="K2" s="142"/>
+      <x:c r="K2" s="234"/>
     </x:row>
     <x:row r="3" s="105" customFormat="1" ht="30" customHeight="1">
-      <x:c r="A3" s="147"/>
-      <x:c r="B3" s="147"/>
-      <x:c r="C3" s="147"/>
-      <x:c r="D3" s="157" t="str">
+      <x:c r="A3" s="238"/>
+      <x:c r="B3" s="238"/>
+      <x:c r="C3" s="238"/>
+      <x:c r="D3" s="238" t="str">
         <x:v>skill-on</x:v>
       </x:c>
-      <x:c r="E3" s="157"/>
-      <x:c r="F3" s="157" t="str">
+      <x:c r="E3" s="238"/>
+      <x:c r="F3" s="238" t="str">
         <x:v>skill-off</x:v>
       </x:c>
-      <x:c r="G3" s="157"/>
-      <x:c r="H3" s="157" t="str">
+      <x:c r="G3" s="238"/>
+      <x:c r="H3" s="238" t="str">
         <x:v>skill-on</x:v>
       </x:c>
-      <x:c r="I3" s="157"/>
-      <x:c r="J3" s="157" t="str">
+      <x:c r="I3" s="238"/>
+      <x:c r="J3" s="238" t="str">
         <x:v>skill-off</x:v>
       </x:c>
-      <x:c r="K3" s="157"/>
+      <x:c r="K3" s="238"/>
     </x:row>
     <x:row r="4" s="105" customFormat="1" ht="30" customHeight="1">
-      <x:c r="A4" s="147"/>
-      <x:c r="B4" s="147"/>
-      <x:c r="C4" s="147"/>
-      <x:c r="D4" s="169" t="str">
+      <x:c r="A4" s="244"/>
+      <x:c r="B4" s="244"/>
+      <x:c r="C4" s="244"/>
+      <x:c r="D4" s="244" t="str">
         <x:v>作答结果</x:v>
       </x:c>
-      <x:c r="E4" s="169" t="str">
+      <x:c r="E4" s="244" t="str">
         <x:v>v0.10.0 得分</x:v>
       </x:c>
-      <x:c r="F4" s="169" t="str">
+      <x:c r="F4" s="244" t="str">
         <x:v>作答结果</x:v>
       </x:c>
-      <x:c r="G4" s="169" t="str">
+      <x:c r="G4" s="244" t="str">
         <x:v>v0.10.0 得分</x:v>
       </x:c>
-      <x:c r="H4" s="169" t="str">
+      <x:c r="H4" s="244" t="str">
         <x:v>作答结果</x:v>
       </x:c>
-      <x:c r="I4" s="169" t="str">
+      <x:c r="I4" s="244" t="str">
         <x:v>v0.10.0 得分</x:v>
       </x:c>
-      <x:c r="J4" s="169" t="str">
+      <x:c r="J4" s="244" t="str">
         <x:v>作答结果</x:v>
       </x:c>
-      <x:c r="K4" s="169" t="str">
+      <x:c r="K4" s="244" t="str">
         <x:v>v0.10.0 得分</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="105" customFormat="1" ht="79.6500015258789" customHeight="1">
-      <x:c r="A5" s="190" t="str">
+      <x:c r="A5" s="252" t="str">
         <x:v>property_calculation_advanced_001_free_energy；概括：计算两种分子晶体在 300 K 时的自由能绝对差。</x:v>
       </x:c>
-      <x:c r="B5" s="191" t="str">
+      <x:c r="B5" s="253" t="str">
         <x:v>±8 kJ/mol</x:v>
       </x:c>
-      <x:c r="C5" s="191" t="str">
+      <x:c r="C5" s="253" t="str">
         <x:v>{"answer":0.258031679,"unit":"kJ/mol"}</x:v>
       </x:c>
-      <x:c r="D5" s="202" t="str">
+      <x:c r="D5" s="256" t="str">
         <x:v>{"answer":0.0799,"unit":"kJ/mol"}</x:v>
       </x:c>
-      <x:c r="E5" s="211" t="n">
+      <x:c r="E5" s="259" t="n">
         <x:v>0.977733540125</x:v>
       </x:c>
-      <x:c r="F5" s="202" t="str">
+      <x:c r="F5" s="256" t="str">
         <x:v>{"answer":90.35,"unit":"kJ/mol"}</x:v>
       </x:c>
-      <x:c r="G5" s="211" t="n">
+      <x:c r="G5" s="259" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H5" s="202" t="str">
+      <x:c r="H5" s="256" t="str">
         <x:v>{"answer":0.08,"unit":"kJ/mol"}</x:v>
       </x:c>
-      <x:c r="I5" s="211" t="n">
+      <x:c r="I5" s="259" t="n">
         <x:v>0.977746040125</x:v>
       </x:c>
-      <x:c r="J5" s="202" t="str">
+      <x:c r="J5" s="256" t="str">
         <x:v>{"answer":2.81,"unit":"kJ/mol"}</x:v>
       </x:c>
-      <x:c r="K5" s="211" t="n">
+      <x:c r="K5" s="259" t="n">
         <x:v>0.681003959875</x:v>
       </x:c>
     </x:row>
     <x:row r="6" s="105" customFormat="1" ht="93.6500015258789" customHeight="1">
-      <x:c r="A6" s="190" t="str">
+      <x:c r="A6" s="252" t="str">
         <x:v>property_calculation_advanced_002_crystal_phase；概括：计算 alpha/beta 晶相势能差并判断常压相和高压相。</x:v>
       </x:c>
-      <x:c r="B6" s="193" t="str">
+      <x:c r="B6" s="252" t="str">
         <x:v>势能差：±0.8 eV；常压相：精确匹配；高压相：精确匹配</x:v>
       </x:c>
-      <x:c r="C6" s="191" t="str">
+      <x:c r="C6" s="253" t="str">
         <x:v>{"answers":[{"property":"potential_energy_difference","value":0.079,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
       </x:c>
-      <x:c r="D6" s="202" t="str">
+      <x:c r="D6" s="256" t="str">
         <x:v>{"answers":[{"property":"potential_energy_difference","value":7.299201259709321,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
       </x:c>
-      <x:c r="E6" s="211" t="n">
+      <x:c r="E6" s="259" t="n">
         <x:v>0.5</x:v>
       </x:c>
-      <x:c r="F6" s="202" t="str">
+      <x:c r="F6" s="256" t="str">
         <x:v>{"answers":[{"property":"potential_energy_difference","value":5.50986,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
       </x:c>
-      <x:c r="G6" s="211" t="n">
+      <x:c r="G6" s="259" t="n">
         <x:v>0.5</x:v>
       </x:c>
-      <x:c r="H6" s="202" t="str">
+      <x:c r="H6" s="256" t="str">
         <x:v>{"answers":[{"property":"potential_energy_difference","value":5.51,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
       </x:c>
-      <x:c r="I6" s="211" t="n">
+      <x:c r="I6" s="259" t="n">
         <x:v>0.5</x:v>
       </x:c>
-      <x:c r="J6" s="202" t="str">
+      <x:c r="J6" s="256" t="str">
         <x:v>{"answers":[{"property":"potential_energy_difference","value":7.17,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
       </x:c>
-      <x:c r="K6" s="211" t="n">
+      <x:c r="K6" s="259" t="n">
         <x:v>0.5</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="105" customFormat="1" ht="76" customHeight="1">
-      <x:c r="A7" s="190" t="str">
+      <x:c r="A7" s="252" t="str">
         <x:v>property_calculation_advanced_003_hbond_count；概括：统计 DEBXIT06 晶体中一个分子参与的氢键总数。</x:v>
       </x:c>
-      <x:c r="B7" s="191" t="str">
+      <x:c r="B7" s="253" t="str">
         <x:v>±2 count</x:v>
       </x:c>
-      <x:c r="C7" s="191" t="str">
+      <x:c r="C7" s="253" t="str">
         <x:v>{"answer":12,"unit":"count"}</x:v>
       </x:c>
-      <x:c r="D7" s="202" t="str">
+      <x:c r="D7" s="256" t="str">
         <x:v>{"answer":12,"unit":"count"}</x:v>
       </x:c>
-      <x:c r="E7" s="211" t="n">
+      <x:c r="E7" s="259" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F7" s="202" t="str">
+      <x:c r="F7" s="256" t="str">
         <x:v>{"answer":12,"unit":"count"}</x:v>
       </x:c>
-      <x:c r="G7" s="211" t="n">
+      <x:c r="G7" s="259" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H7" s="202" t="str">
+      <x:c r="H7" s="256" t="str">
         <x:v>{"answer":12,"unit":"count"}</x:v>
       </x:c>
-      <x:c r="I7" s="211" t="n">
+      <x:c r="I7" s="259" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J7" s="202" t="str">
+      <x:c r="J7" s="256" t="str">
         <x:v>{"answer":10,"unit":"count"}</x:v>
       </x:c>
-      <x:c r="K7" s="211" t="n">
+      <x:c r="K7" s="259" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="105" customFormat="1" ht="92.05000305175781" customHeight="1">
-      <x:c r="A8" s="190" t="str">
+      <x:c r="A8" s="252" t="str">
         <x:v>property_calculation_advanced_004_ir_top2_frequencies；概括：给出最低能白藜芦醇构象中 IR 强度最大的两个振动频率。</x:v>
       </x:c>
-      <x:c r="B8" s="191" t="str">
+      <x:c r="B8" s="253" t="str">
         <x:v>频率1：±100 cm^-1；频率2：±100 cm^-1</x:v>
       </x:c>
-      <x:c r="C8" s="191" t="str">
+      <x:c r="C8" s="253" t="str">
         <x:v>{"answers":[{"property":"frequency_1","value":1208.10,"unit":"cm^-1"},{"property":"frequency_2","value":1685.56,"unit":"cm^-1"}]}</x:v>
       </x:c>
-      <x:c r="D8" s="202" t="str">
+      <x:c r="D8" s="256" t="str">
         <x:v>{"answers":[{"property":"frequency_1","value":435.81,"unit":"cm^-1"},{"property":"frequency_2","value":1585.74,"unit":"cm^-1"},{"property":"frequency_3","value":1592.57,"unit":"cm^-1"}]}</x:v>
       </x:c>
-      <x:c r="E8" s="211" t="n">
+      <x:c r="E8" s="259" t="n">
         <x:v>0.000900000000000345</x:v>
       </x:c>
-      <x:c r="F8" s="202" t="str">
+      <x:c r="F8" s="256" t="str">
         <x:v>{"answers":[{"property":"frequency_1","value":1585.71,"unit":"cm^-1"},{"property":"frequency_2","value":436.11,"unit":"cm^-1"},{"property":"frequency_3","value":1592.37,"unit":"cm^-1"}]}</x:v>
       </x:c>
-      <x:c r="G8" s="211" t="n">
+      <x:c r="G8" s="259" t="n">
         <x:v>0.0007500000000004725</x:v>
       </x:c>
-      <x:c r="H8" s="202" t="str">
+      <x:c r="H8" s="256" t="str">
         <x:v>{"answers":[{"property":"frequency_1","value":1584.79,"unit":"cm^-1"},{"property":"frequency_2","value":433.87,"unit":"cm^-1"},{"property":"frequency_3","value":1592.2,"unit":"cm^-1"}]}</x:v>
       </x:c>
-      <x:c r="I8" s="211" t="n">
+      <x:c r="I8" s="259" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J8" s="202" t="str">
+      <x:c r="J8" s="256" t="str">
         <x:v>{"answers":[{"property":"frequency_1","value":1624.6,"unit":"cm^-1"},{"property":"frequency_2","value":1246.4,"unit":"cm^-1"},{"property":"frequency_3","value":843.1,"unit":"cm^-1"}]}</x:v>
       </x:c>
-      <x:c r="K8" s="211" t="n">
+      <x:c r="K8" s="259" t="n">
         <x:v>0.5036999999999989</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="105" customFormat="1" ht="76" customHeight="1">
-      <x:c r="A9" s="190" t="str">
+      <x:c r="A9" s="252" t="str">
         <x:v>property_calculation_advanced_005_crystal_density；概括：估算咖啡因一水合物晶体的密度。</x:v>
       </x:c>
-      <x:c r="B9" s="191" t="str">
+      <x:c r="B9" s="253" t="str">
         <x:v>±10%</x:v>
       </x:c>
-      <x:c r="C9" s="191" t="str">
+      <x:c r="C9" s="253" t="str">
         <x:v>{"answer":1.44728,"unit":"g/cm^3"}</x:v>
       </x:c>
-      <x:c r="D9" s="202" t="str">
+      <x:c r="D9" s="256" t="str">
         <x:v>{"answer":1.55,"unit":"g/cm^3"}</x:v>
       </x:c>
-      <x:c r="E9" s="211" t="n">
+      <x:c r="E9" s="259" t="n">
         <x:v>0.2902548228400852</x:v>
       </x:c>
-      <x:c r="F9" s="202" t="str">
+      <x:c r="F9" s="256" t="str">
         <x:v>{"answer":1.56,"unit":"g/cm^3"}</x:v>
       </x:c>
-      <x:c r="G9" s="211" t="n">
+      <x:c r="G9" s="259" t="n">
         <x:v>0.2211596926648599</x:v>
       </x:c>
-      <x:c r="H9" s="202" t="str">
+      <x:c r="H9" s="256" t="str">
         <x:v>{"answer":1.47,"unit":"g/cm^3"}</x:v>
       </x:c>
-      <x:c r="I9" s="211" t="n">
+      <x:c r="I9" s="259" t="n">
         <x:v>0.8430158642418877</x:v>
       </x:c>
-      <x:c r="J9" s="202" t="str">
+      <x:c r="J9" s="256" t="str">
         <x:v>{"answer":1.28,"unit":"g/cm^3"}</x:v>
       </x:c>
-      <x:c r="K9" s="211" t="n">
+      <x:c r="K9" s="259" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="10" s="105" customFormat="1" ht="76" customHeight="1">
-      <x:c r="A10" s="190" t="str">
+      <x:c r="A10" s="252" t="str">
         <x:v>property_calculation_advanced_006_cocrystal_ratio；概括：确定大麻酚与四甲基吡嗪在最终共晶中的摩尔比。</x:v>
       </x:c>
-      <x:c r="B10" s="191" t="str">
+      <x:c r="B10" s="253" t="str">
         <x:v>精确匹配</x:v>
       </x:c>
-      <x:c r="C10" s="191" t="str">
+      <x:c r="C10" s="253" t="str">
         <x:v>{"answer":"1:1"}</x:v>
       </x:c>
-      <x:c r="D10" s="202" t="str">
+      <x:c r="D10" s="256" t="str">
         <x:v>{"answer":"1:1"}</x:v>
       </x:c>
-      <x:c r="E10" s="211" t="n">
+      <x:c r="E10" s="259" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F10" s="202" t="str">
+      <x:c r="F10" s="256" t="str">
         <x:v>{"answer":"1:1"}</x:v>
       </x:c>
-      <x:c r="G10" s="211" t="n">
+      <x:c r="G10" s="259" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H10" s="202" t="str">
+      <x:c r="H10" s="256" t="str">
         <x:v>{"answer":"1:1"}</x:v>
       </x:c>
-      <x:c r="I10" s="211" t="n">
+      <x:c r="I10" s="259" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J10" s="202" t="str">
+      <x:c r="J10" s="256" t="str">
         <x:v>{"answer":"1:2"}</x:v>
       </x:c>
-      <x:c r="K10" s="211" t="n">
+      <x:c r="K10" s="259" t="n">
         <x:v>0.5</x:v>
       </x:c>
     </x:row>
     <x:row r="11" s="105" customFormat="1" ht="76" customHeight="1">
-      <x:c r="A11" s="190" t="str">
+      <x:c r="A11" s="252" t="str">
         <x:v>property_calculation_advanced_007_polymorph_free_energy_crossover；概括：判断 Radiprodil FormA/FormC 在 0 K 的低自由能晶型及交叉温度。</x:v>
       </x:c>
-      <x:c r="B11" s="191" t="str">
+      <x:c r="B11" s="253" t="str">
         <x:v>0 K 低自由能晶型：精确匹配；交叉温度：±100 K</x:v>
       </x:c>
-      <x:c r="C11" s="191" t="str">
+      <x:c r="C11" s="253" t="str">
         <x:v>{"answers":[{"property":"lower_free_energy_at_0k","value":"FormC"},{"property":"crossover_temperature","value":343.15,"unit":"K"}]}</x:v>
       </x:c>
-      <x:c r="D11" s="202" t="str">
+      <x:c r="D11" s="256" t="str">
         <x:v>{"answers":[{"property":"lower_free_energy_at_0k","value":"FormA"},{"property":"crossover_temperature","value":3016,"unit":"K"}]}</x:v>
       </x:c>
-      <x:c r="E11" s="211" t="n">
+      <x:c r="E11" s="259" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F11" s="202" t="str">
+      <x:c r="F11" s="256" t="str">
         <x:v>{"answers":[{"property":"lower_free_energy_at_0k","value":"FormC"},{"property":"crossover_temperature","value":943,"unit":"K"}]}</x:v>
       </x:c>
-      <x:c r="G11" s="211" t="n">
+      <x:c r="G11" s="259" t="n">
         <x:v>0.5</x:v>
       </x:c>
-      <x:c r="H11" s="202" t="str">
+      <x:c r="H11" s="256" t="str">
         <x:v>{"answers":[{"property":"lower_free_energy_at_0k","value":"FormA"},{"property":"crossover_temperature","value":428.5,"unit":"K"}]}</x:v>
       </x:c>
-      <x:c r="I11" s="211" t="n">
+      <x:c r="I11" s="259" t="n">
         <x:v>0.07324999999999987</x:v>
       </x:c>
-      <x:c r="J11" s="202" t="str">
+      <x:c r="J11" s="256" t="str">
         <x:v>{"answers":[{"property":"lower_free_energy_at_0k","value":"FormA"},{"property":"crossover_temperature","value":300,"unit":"K"}]}</x:v>
       </x:c>
-      <x:c r="K11" s="211" t="n">
+      <x:c r="K11" s="259" t="n">
         <x:v>0.2842500000000001</x:v>
       </x:c>
     </x:row>
     <x:row r="12" s="105" customFormat="1" ht="76" customHeight="1">
-      <x:c r="A12" s="190" t="str">
+      <x:c r="A12" s="252" t="str">
         <x:v>property_calculation_advanced_008_interaction_binding_energy；概括：计算指定二聚体的相互作用能和结合能并保留符号。</x:v>
       </x:c>
-      <x:c r="B12" s="191" t="str">
+      <x:c r="B12" s="253" t="str">
         <x:v>相互作用能：±10 kcal/mol；结合能：±10 kcal/mol</x:v>
       </x:c>
-      <x:c r="C12" s="191" t="str">
+      <x:c r="C12" s="253" t="str">
         <x:v>{"answers":[{"property":"interaction_energy","value":-69.04,"unit":"kcal/mol"},{"property":"binding_energy","value":-58.15,"unit":"kcal/mol"}]}</x:v>
       </x:c>
-      <x:c r="D12" s="202" t="str">
+      <x:c r="D12" s="256" t="str">
         <x:v>{"answers":[{"property":"interaction_energy","value":-70.4733,"unit":"kcal/mol"},{"property":"binding_energy","value":-59.3678,"unit":"kcal/mol"}]}</x:v>
       </x:c>
-      <x:c r="E12" s="211" t="n">
+      <x:c r="E12" s="259" t="n">
         <x:v>0.8674450000000004</x:v>
       </x:c>
-      <x:c r="F12" s="202" t="str">
+      <x:c r="F12" s="256" t="str">
         <x:v>{"answers":[{"property":"interaction_energy","value":-70.47,"unit":"kcal/mol"},{"property":"binding_energy","value":-59.38,"unit":"kcal/mol"}]}</x:v>
       </x:c>
-      <x:c r="G12" s="211" t="n">
+      <x:c r="G12" s="259" t="n">
         <x:v>0.8670000000000002</x:v>
       </x:c>
-      <x:c r="H12" s="202" t="str">
+      <x:c r="H12" s="256" t="str">
         <x:v>{"answers":[{"property":"interaction_energy","value":-70.45,"unit":"kcal/mol"},{"property":"binding_energy","value":-59.37,"unit":"kcal/mol"}]}</x:v>
       </x:c>
-      <x:c r="I12" s="211" t="n">
+      <x:c r="I12" s="259" t="n">
         <x:v>0.8685000000000003</x:v>
       </x:c>
-      <x:c r="J12" s="202" t="str">
+      <x:c r="J12" s="256" t="str">
         <x:v>{"answers":[{"property":"interaction_energy","value":-70.49,"unit":"kcal/mol"},{"property":"binding_energy","value":-59.38,"unit":"kcal/mol"}]}</x:v>
       </x:c>
-      <x:c r="K12" s="211" t="n">
+      <x:c r="K12" s="259" t="n">
         <x:v>0.8660000000000003</x:v>
       </x:c>
     </x:row>
     <x:row r="13" s="105" customFormat="1" ht="76" customHeight="1">
-      <x:c r="A13" s="190" t="str">
+      <x:c r="A13" s="252" t="str">
         <x:v>property_calculation_advanced_009_homo_lumo_gap；概括：计算指定分子的 HOMO-LUMO 能隙。</x:v>
       </x:c>
-      <x:c r="B13" s="191" t="str">
+      <x:c r="B13" s="253" t="str">
         <x:v>±1 eV</x:v>
       </x:c>
-      <x:c r="C13" s="191" t="str">
+      <x:c r="C13" s="253" t="str">
         <x:v>{"answer":7.26,"unit":"eV"}</x:v>
       </x:c>
-      <x:c r="D13" s="202" t="str">
+      <x:c r="D13" s="256" t="str">
         <x:v>{"answer":3.558797467914,"unit":"eV"}</x:v>
       </x:c>
-      <x:c r="E13" s="211" t="n">
+      <x:c r="E13" s="259" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F13" s="202" t="str">
+      <x:c r="F13" s="256" t="str">
         <x:v>{"answer":3.559175368755,"unit":"eV"}</x:v>
       </x:c>
-      <x:c r="G13" s="211" t="n">
+      <x:c r="G13" s="259" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H13" s="202" t="str">
+      <x:c r="H13" s="256" t="str">
         <x:v>{"answer":3.5845,"unit":"eV"}</x:v>
       </x:c>
-      <x:c r="I13" s="211" t="n">
+      <x:c r="I13" s="259" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J13" s="202" t="str">
+      <x:c r="J13" s="256" t="str">
         <x:v>{"answer":3.584,"unit":"eV"}</x:v>
       </x:c>
-      <x:c r="K13" s="211" t="n">
+      <x:c r="K13" s="259" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="14" s="105" customFormat="1" ht="76" customHeight="1">
-      <x:c r="A14" s="190" t="str">
+      <x:c r="A14" s="252" t="str">
         <x:v>property_calculation_advanced_010_hbond_distances；概括：计算尿素-磷酸相互作用单元的 O-H 键长与 H...O 接触距离。</x:v>
       </x:c>
-      <x:c r="B14" s="191" t="str">
+      <x:c r="B14" s="253" t="str">
         <x:v>O–H 键距：±0.1 Å；H···O 接触距离：±0.1 Å</x:v>
       </x:c>
-      <x:c r="C14" s="191" t="str">
+      <x:c r="C14" s="253" t="str">
         <x:v>{"answers":[{"property":"oh_bond_distance","value":1.029,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.485,"unit":"angstrom"}]}</x:v>
       </x:c>
-      <x:c r="D14" s="202" t="str">
+      <x:c r="D14" s="256" t="str">
         <x:v>{"answers":[{"property":"oh_bond_distance","value":1.002,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.592,"unit":"angstrom"}]}</x:v>
       </x:c>
-      <x:c r="E14" s="211" t="n">
+      <x:c r="E14" s="259" t="n">
         <x:v>0.36500000000000044</x:v>
       </x:c>
-      <x:c r="F14" s="202" t="str">
+      <x:c r="F14" s="256" t="str">
         <x:v>{"answers":[{"property":"oh_bond_distance","value":1.001520301,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.594671850,"unit":"angstrom"}]}</x:v>
       </x:c>
-      <x:c r="G14" s="211" t="n">
+      <x:c r="G14" s="259" t="n">
         <x:v>0.36260150500000043</x:v>
       </x:c>
-      <x:c r="H14" s="202" t="str">
+      <x:c r="H14" s="256" t="str">
         <x:v>{"answers":[{"property":"oh_bond_distance","value":1.002,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.592,"unit":"angstrom"}]}</x:v>
       </x:c>
-      <x:c r="I14" s="211" t="n">
+      <x:c r="I14" s="259" t="n">
         <x:v>0.36500000000000044</x:v>
       </x:c>
-      <x:c r="J14" s="202" t="str">
+      <x:c r="J14" s="256" t="str">
         <x:v>{"answers":[{"property":"oh_bond_distance","value":1.002,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.592,"unit":"angstrom"}]}</x:v>
       </x:c>
-      <x:c r="K14" s="211" t="n">
+      <x:c r="K14" s="259" t="n">
         <x:v>0.36500000000000044</x:v>
       </x:c>
     </x:row>
     <x:row r="15" s="105" customFormat="1" ht="76" customHeight="1">
-      <x:c r="A15" s="190" t="str">
+      <x:c r="A15" s="252" t="str">
         <x:v>property_calculation_advanced_011_accessible_pore_volume_ratio；概括：计算 NOGCOE 晶胞的可达体积与不可达体积之比。</x:v>
       </x:c>
-      <x:c r="B15" s="191" t="str">
+      <x:c r="B15" s="253" t="str">
         <x:v>±0.5</x:v>
       </x:c>
-      <x:c r="C15" s="191" t="str">
+      <x:c r="C15" s="253" t="str">
         <x:v>{"answer":1.713,"unit":"ratio"}</x:v>
       </x:c>
-      <x:c r="D15" s="202" t="str">
+      <x:c r="D15" s="256" t="str">
         <x:v>{"answer":0.0443,"unit":"ratio"}</x:v>
       </x:c>
-      <x:c r="E15" s="211" t="n">
+      <x:c r="E15" s="259" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F15" s="202" t="str">
+      <x:c r="F15" s="256" t="str">
         <x:v>{"answer":0.07236,"unit":"ratio"}</x:v>
       </x:c>
-      <x:c r="G15" s="211" t="n">
+      <x:c r="G15" s="259" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H15" s="202" t="str">
+      <x:c r="H15" s="256" t="str">
         <x:v>{"answer":0.076,"unit":"ratio"}</x:v>
       </x:c>
-      <x:c r="I15" s="211" t="n">
+      <x:c r="I15" s="259" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J15" s="202" t="str">
+      <x:c r="J15" s="256" t="str">
         <x:v>{"answer":0.0724,"unit":"ratio"}</x:v>
       </x:c>
-      <x:c r="K15" s="211" t="n">
+      <x:c r="K15" s="259" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="16" s="105" customFormat="1" ht="76" customHeight="1">
-      <x:c r="A16" s="190" t="str">
+      <x:c r="A16" s="252" t="str">
         <x:v>property_calculation_advanced_012_carboxyl_hydrogen_distance；概括：计算指定二羧酸最低能构象中两个羧酸氢的距离。</x:v>
       </x:c>
-      <x:c r="B16" s="191" t="str">
+      <x:c r="B16" s="253" t="str">
         <x:v>±0.2 Å</x:v>
       </x:c>
-      <x:c r="C16" s="191" t="str">
+      <x:c r="C16" s="253" t="str">
         <x:v>{"answer":2.521,"unit":"angstrom"}</x:v>
       </x:c>
-      <x:c r="D16" s="202" t="str">
+      <x:c r="D16" s="256" t="str">
         <x:v>{"answer":2.5212,"unit":"angstrom"}</x:v>
       </x:c>
-      <x:c r="E16" s="211" t="n">
+      <x:c r="E16" s="259" t="n">
         <x:v>0.9990000000000001</x:v>
       </x:c>
-      <x:c r="F16" s="202" t="str">
+      <x:c r="F16" s="256" t="str">
         <x:v>{"answer":2.5183,"unit":"angstrom"}</x:v>
       </x:c>
-      <x:c r="G16" s="211" t="n">
+      <x:c r="G16" s="259" t="n">
         <x:v>0.9865000000000004</x:v>
       </x:c>
-      <x:c r="H16" s="202" t="str">
+      <x:c r="H16" s="256" t="str">
         <x:v>{"answer":2.52,"unit":"angstrom"}</x:v>
       </x:c>
-      <x:c r="I16" s="211" t="n">
+      <x:c r="I16" s="259" t="n">
         <x:v>0.9950000000000006</x:v>
       </x:c>
-      <x:c r="J16" s="202" t="str">
+      <x:c r="J16" s="256" t="str">
         <x:v>{"answer":2.7043,"unit":"angstrom"}</x:v>
       </x:c>
-      <x:c r="K16" s="211" t="n">
+      <x:c r="K16" s="259" t="n">
         <x:v>0.08349999999999991</x:v>
       </x:c>
     </x:row>
     <x:row r="17" s="105" customFormat="1" ht="76" customHeight="1">
-      <x:c r="A17" s="190" t="str">
+      <x:c r="A17" s="252" t="str">
         <x:v>property_calculation_advanced_013_halogen_bond_energy；概括：计算 FI...NH3 卤键复合物的相互作用能并保留符号。</x:v>
       </x:c>
-      <x:c r="B17" s="191" t="str">
+      <x:c r="B17" s="253" t="str">
         <x:v>±5 kcal/mol</x:v>
       </x:c>
-      <x:c r="C17" s="191" t="str">
+      <x:c r="C17" s="253" t="str">
         <x:v>{"answer":-17.11,"unit":"kcal/mol"}</x:v>
       </x:c>
-      <x:c r="D17" s="202" t="str">
+      <x:c r="D17" s="256" t="str">
         <x:v>{"answer":-17.11,"unit":"kcal/mol"}</x:v>
       </x:c>
-      <x:c r="E17" s="211" t="n">
+      <x:c r="E17" s="259" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F17" s="202" t="str">
+      <x:c r="F17" s="256" t="str">
         <x:v>{"answer":-19.17,"unit":"kcal/mol"}</x:v>
       </x:c>
-      <x:c r="G17" s="211" t="n">
+      <x:c r="G17" s="259" t="n">
         <x:v>0.5879999999999995</x:v>
       </x:c>
-      <x:c r="H17" s="202" t="str">
+      <x:c r="H17" s="256" t="str">
         <x:v>{"answer":-15.5969,"unit":"kcal/mol"}</x:v>
       </x:c>
-      <x:c r="I17" s="211" t="n">
+      <x:c r="I17" s="259" t="n">
         <x:v>0.6973800000000001</x:v>
       </x:c>
-      <x:c r="J17" s="202" t="str">
+      <x:c r="J17" s="256" t="str">
         <x:v>{"answer":-16.5,"unit":"kcal/mol"}</x:v>
       </x:c>
-      <x:c r="K17" s="211" t="n">
+      <x:c r="K17" s="259" t="n">
         <x:v>0.8780000000000001</x:v>
       </x:c>
     </x:row>
     <x:row r="18" s="105" customFormat="1" ht="76" customHeight="1">
-      <x:c r="A18" s="190" t="str">
+      <x:c r="A18" s="252" t="str">
         <x:v>property_calculation_advanced_014_bay069_pka；概括：计算 BAY-069 分子的 pKa。</x:v>
       </x:c>
-      <x:c r="B18" s="191" t="str">
+      <x:c r="B18" s="253" t="str">
         <x:v>±2 pKa</x:v>
       </x:c>
-      <x:c r="C18" s="191" t="str">
+      <x:c r="C18" s="253" t="str">
         <x:v>{"answer":5.7,"unit":"pKa"}</x:v>
       </x:c>
-      <x:c r="D18" s="202" t="str">
+      <x:c r="D18" s="256" t="str">
         <x:v>{"answer":5.0,"unit":"pKa"}</x:v>
       </x:c>
-      <x:c r="E18" s="211" t="n">
+      <x:c r="E18" s="259" t="n">
         <x:v>0.6499999999999999</x:v>
       </x:c>
-      <x:c r="F18" s="202" t="str">
+      <x:c r="F18" s="256" t="str">
         <x:v>{"answer":6.33,"unit":"pKa"}</x:v>
       </x:c>
-      <x:c r="G18" s="211" t="n">
+      <x:c r="G18" s="259" t="n">
         <x:v>0.685</x:v>
       </x:c>
-      <x:c r="H18" s="202" t="str">
+      <x:c r="H18" s="256" t="str">
         <x:v>{"answer":5.7,"unit":"pKa"}</x:v>
       </x:c>
-      <x:c r="I18" s="211" t="n">
+      <x:c r="I18" s="259" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J18" s="202" t="str">
+      <x:c r="J18" s="256" t="str">
         <x:v>{"answer":6.8,"unit":"pKa"}</x:v>
       </x:c>
-      <x:c r="K18" s="211" t="n">
+      <x:c r="K18" s="259" t="n">
         <x:v>0.4500000000000002</x:v>
       </x:c>
     </x:row>
     <x:row r="19" s="105" customFormat="1" ht="76" customHeight="1">
-      <x:c r="A19" s="190" t="str">
+      <x:c r="A19" s="252" t="str">
         <x:v>property_calculation_advanced_015_formaldehyde_socme；概括：计算气相甲醛 T1-S0 自旋轨道耦合矩阵元的大小。</x:v>
       </x:c>
-      <x:c r="B19" s="191" t="str">
+      <x:c r="B19" s="253" t="str">
         <x:v>±1 log10（数量级）</x:v>
       </x:c>
-      <x:c r="C19" s="191" t="str">
+      <x:c r="C19" s="253" t="str">
         <x:v>{"answer":0.00734,"unit":"eV"}</x:v>
       </x:c>
-      <x:c r="D19" s="202" t="str">
+      <x:c r="D19" s="256" t="str">
         <x:v>{"answer":0.00485,"unit":"eV"}</x:v>
       </x:c>
-      <x:c r="E19" s="211" t="n">
+      <x:c r="E19" s="259" t="n">
         <x:v>0.8200456786861929</x:v>
       </x:c>
-      <x:c r="F19" s="202" t="str">
+      <x:c r="F19" s="256" t="str">
         <x:v>{"answer":0.0035,"unit":"eV"}</x:v>
       </x:c>
-      <x:c r="G19" s="211" t="n">
+      <x:c r="G19" s="259" t="n">
         <x:v>0.6783719844342051</x:v>
       </x:c>
-      <x:c r="H19" s="202" t="str">
+      <x:c r="H19" s="256" t="str">
         <x:v>{"answer":0.0,"unit":"eV"}</x:v>
       </x:c>
-      <x:c r="I19" s="211" t="n">
+      <x:c r="I19" s="259" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J19" s="202" t="str">
+      <x:c r="J19" s="256" t="str">
         <x:v>{"answer":0.01,"unit":"eV"}</x:v>
       </x:c>
-      <x:c r="K19" s="211" t="n">
+      <x:c r="K19" s="259" t="n">
         <x:v>0.8656960599160706</x:v>
       </x:c>
     </x:row>
     <x:row r="20" s="105" customFormat="1" ht="76" customHeight="1">
-      <x:c r="A20" s="190" t="str">
+      <x:c r="A20" s="252" t="str">
         <x:v>property_calculation_advanced_016_anthracene_isc_rate；概括：计算气相蒽在 77 K 的 S1 系间窜越速率常数。</x:v>
       </x:c>
-      <x:c r="B20" s="191" t="str">
+      <x:c r="B20" s="253" t="str">
         <x:v>±2 log10（数量级）</x:v>
       </x:c>
-      <x:c r="C20" s="191" t="str">
+      <x:c r="C20" s="253" t="str">
         <x:v>{"answer":117000000,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="D20" s="202" t="str">
+      <x:c r="D20" s="256" t="str">
         <x:v>{"answer":1.2e8,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="E20" s="211" t="n">
+      <x:c r="E20" s="259" t="n">
         <x:v>0.9945023078492685</x:v>
       </x:c>
-      <x:c r="F20" s="202" t="str">
+      <x:c r="F20" s="256" t="str">
         <x:v>{"answer":1.45e8,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="G20" s="211" t="n">
+      <x:c r="G20" s="259" t="n">
         <x:v>0.9534089297555939</x:v>
       </x:c>
-      <x:c r="H20" s="202" t="str">
+      <x:c r="H20" s="256" t="str">
         <x:v>{"answer":1e6,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="I20" s="211" t="n">
+      <x:c r="I20" s="259" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J20" s="202" t="str">
+      <x:c r="J20" s="256" t="str">
         <x:v>{"answer":100000,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="K20" s="211" t="n">
+      <x:c r="K20" s="259" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="21" s="105" customFormat="1" ht="79.4000015258789" customHeight="1">
-      <x:c r="A21" s="190" t="str">
+      <x:c r="A21" s="252" t="str">
         <x:v>property_calculation_advanced_017_biacetyl_phosphorescence_rate；概括：计算乙醇隐式溶剂中联乙酰在 298 K 的磷光速率常数。</x:v>
       </x:c>
-      <x:c r="B21" s="191" t="str">
+      <x:c r="B21" s="253" t="str">
         <x:v>±2 log10（数量级）</x:v>
       </x:c>
-      <x:c r="C21" s="191" t="str">
+      <x:c r="C21" s="253" t="str">
         <x:v>{"answer":98,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="D21" s="202" t="str">
+      <x:c r="D21" s="256" t="str">
         <x:v>{"answer":91.92785,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="E21" s="211" t="n">
+      <x:c r="E21" s="259" t="n">
         <x:v>0.9861105136520333</x:v>
       </x:c>
-      <x:c r="F21" s="202" t="str">
+      <x:c r="F21" s="256" t="str">
         <x:v>{"answer":100.0,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="G21" s="211" t="n">
+      <x:c r="G21" s="259" t="n">
         <x:v>0.9956130378462474</x:v>
       </x:c>
-      <x:c r="H21" s="202" t="str">
+      <x:c r="H21" s="256" t="str">
         <x:v>{"answer":100,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="I21" s="211" t="n">
+      <x:c r="I21" s="259" t="n">
         <x:v>0.9956130378462474</x:v>
       </x:c>
-      <x:c r="J21" s="202" t="str">
+      <x:c r="J21" s="256" t="str">
         <x:v>{"answer":16.9,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="K21" s="211" t="n">
+      <x:c r="K21" s="259" t="n">
         <x:v>0.6183303144605893</x:v>
       </x:c>
     </x:row>
     <x:row r="22" s="105" customFormat="1" ht="76" customHeight="1">
-      <x:c r="A22" s="190" t="str">
+      <x:c r="A22" s="252" t="str">
         <x:v>property_calculation_advanced_018_anthracene_ht_contribution；概括：计算气相蒽在 77 K 的 Herzberg-Teller 项对 S1-T1 系间窜越速率的贡献比例。</x:v>
       </x:c>
-      <x:c r="B22" s="191" t="str">
+      <x:c r="B22" s="253" t="str">
         <x:v>−10/+1 %</x:v>
       </x:c>
-      <x:c r="C22" s="191" t="str">
+      <x:c r="C22" s="253" t="str">
         <x:v>{"answer":100,"unit":"percent"}</x:v>
       </x:c>
-      <x:c r="D22" s="202" t="str">
+      <x:c r="D22" s="256" t="str">
         <x:v>{"answer":100,"unit":"percent"}</x:v>
       </x:c>
-      <x:c r="E22" s="211" t="n">
+      <x:c r="E22" s="259" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F22" s="202" t="str">
+      <x:c r="F22" s="256" t="str">
         <x:v>{"answer":70,"unit":"percent"}</x:v>
       </x:c>
-      <x:c r="G22" s="211" t="n">
+      <x:c r="G22" s="259" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H22" s="202" t="str">
+      <x:c r="H22" s="256" t="str">
         <x:v>{"answer":100,"unit":"percent"}</x:v>
       </x:c>
-      <x:c r="I22" s="211" t="n">
+      <x:c r="I22" s="259" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J22" s="202" t="str">
+      <x:c r="J22" s="256" t="str">
         <x:v>{"answer":100,"unit":"percent"}</x:v>
       </x:c>
-      <x:c r="K22" s="211" t="n">
+      <x:c r="K22" s="259" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="23" s="105" customFormat="1" ht="79.4000015258789" customHeight="1">
-      <x:c r="A23" s="190" t="str">
+      <x:c r="A23" s="252" t="str">
         <x:v>property_calculation_advanced_019_acetophenone_isc_rate；概括：计算气相苯乙酮在 77 K 含 Herzberg-Teller 效应的 S1-T1 系间窜越速率。</x:v>
       </x:c>
-      <x:c r="B23" s="191" t="str">
+      <x:c r="B23" s="253" t="str">
         <x:v>±2 log10（数量级）</x:v>
       </x:c>
-      <x:c r="C23" s="191" t="str">
+      <x:c r="C23" s="253" t="str">
         <x:v>{"answer":28400000000,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="D23" s="202" t="str">
+      <x:c r="D23" s="256" t="str">
         <x:v>{"answer":2.38e10,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="E23" s="211" t="n">
+      <x:c r="E23" s="259" t="n">
         <x:v>0.9616293085047376</x:v>
       </x:c>
-      <x:c r="F23" s="202" t="str">
+      <x:c r="F23" s="256" t="str">
         <x:v>{"answer":1.6e8,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="G23" s="211" t="n">
+      <x:c r="G23" s="259" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H23" s="202" t="str">
+      <x:c r="H23" s="256" t="str">
         <x:v>{"answer":1e10,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="I23" s="211" t="n">
+      <x:c r="I23" s="259" t="n">
         <x:v>0.7733408299764815</x:v>
       </x:c>
-      <x:c r="J23" s="202" t="str">
+      <x:c r="J23" s="256" t="str">
         <x:v>{"answer":1e10,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="K23" s="211" t="n">
+      <x:c r="K23" s="259" t="n">
         <x:v>0.7733408299764815</x:v>
       </x:c>
     </x:row>
     <x:row r="24" s="105" customFormat="1" ht="76" customHeight="1">
-      <x:c r="A24" s="190" t="str">
+      <x:c r="A24" s="252" t="str">
         <x:v>property_calculation_advanced_020_azulene_internal_conversion_rate；概括：计算甲醇隐式溶剂中薁在 298.15 K 的 S1-S0 内转换速率。</x:v>
       </x:c>
-      <x:c r="B24" s="191" t="str">
+      <x:c r="B24" s="253" t="str">
         <x:v>±2 log10（数量级）</x:v>
       </x:c>
-      <x:c r="C24" s="191" t="str">
+      <x:c r="C24" s="253" t="str">
         <x:v>{"answer":382000000,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="D24" s="202" t="str">
+      <x:c r="D24" s="256" t="str">
         <x:v>{"answer":1e12,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="E24" s="211" t="n">
+      <x:c r="E24" s="259" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F24" s="202" t="str">
+      <x:c r="F24" s="256" t="str">
         <x:v>{"answer":9.4e11,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="G24" s="211" t="n">
+      <x:c r="G24" s="259" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H24" s="202" t="str">
+      <x:c r="H24" s="256" t="str">
         <x:v>{"answer":1.0e9,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="I24" s="211" t="n">
+      <x:c r="I24" s="259" t="n">
         <x:v>0.7910316814558547</x:v>
       </x:c>
-      <x:c r="J24" s="202"/>
-      <x:c r="K24" s="211" t="n">
+      <x:c r="J24" s="256"/>
+      <x:c r="K24" s="259" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="25" s="105" customFormat="1" ht="28" customHeight="1">
-      <x:c r="A25" s="215" t="str">
+      <x:c r="A25" s="262" t="str">
         <x:v>各实验组平均分（未评分项记0分）</x:v>
       </x:c>
-      <x:c r="B25" s="222"/>
-      <x:c r="C25" s="222"/>
-      <x:c r="D25" s="221" t="str">
+      <x:c r="B25" s="265"/>
+      <x:c r="C25" s="265"/>
+      <x:c r="D25" s="268" t="str">
         <x:v>平均分</x:v>
       </x:c>
-      <x:c r="E25" s="221" t="n">
+      <x:c r="E25" s="268" t="n">
         <x:v>0.6206310585828658</x:v>
       </x:c>
-      <x:c r="F25" s="221" t="str">
+      <x:c r="F25" s="268" t="str">
         <x:v>平均分</x:v>
       </x:c>
-      <x:c r="G25" s="221" t="n">
+      <x:c r="G25" s="268" t="n">
         <x:v>0.4669202574850454</x:v>
       </x:c>
-      <x:c r="H25" s="221" t="str">
+      <x:c r="H25" s="268" t="str">
         <x:v>平均分</x:v>
       </x:c>
-      <x:c r="I25" s="221" t="n">
+      <x:c r="I25" s="268" t="n">
         <x:v>0.5939938726822735</x:v>
       </x:c>
-      <x:c r="J25" s="221" t="str">
+      <x:c r="J25" s="268" t="str">
         <x:v>平均分</x:v>
       </x:c>
-      <x:c r="K25" s="221" t="n">
+      <x:c r="K25" s="268" t="n">
         <x:v>0.41844105821140704</x:v>
       </x:c>
     </x:row>

</xml_diff>